<commit_message>
file downloads done, uses alt if main url fails
</commit_message>
<xml_diff>
--- a/pdf_downloader/src/input/testfile.xlsx
+++ b/pdf_downloader/src/input/testfile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnar Marinosonn\Documents\pdfDownloader\PdfDownloader\pdf_downloader\src\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A115E99-58B2-4B34-ADDC-B5975C3C1051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0A6D7A-0AE5-4FA4-A495-B3E2DC265715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41A94F23-48B9-421F-8120-50C347710791}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11175" xr2:uid="{41A94F23-48B9-421F-8120-50C347710791}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>id</t>
   </si>
@@ -497,6 +497,9 @@
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6">

</xml_diff>

<commit_message>
excel output done, reset functionality added. cli input added
</commit_message>
<xml_diff>
--- a/pdf_downloader/src/input/testfile.xlsx
+++ b/pdf_downloader/src/input/testfile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnar Marinosonn\Documents\pdfDownloader\PdfDownloader\pdf_downloader\src\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0A6D7A-0AE5-4FA4-A495-B3E2DC265715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3547E0-775E-4EB6-B661-777868310850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11175" xr2:uid="{41A94F23-48B9-421F-8120-50C347710791}"/>
+    <workbookView xWindow="3120" yWindow="870" windowWidth="24735" windowHeight="13425" xr2:uid="{41A94F23-48B9-421F-8120-50C347710791}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>